<commit_message>
puzzles: add topology bead loops and tighten cube removal
</commit_message>
<xml_diff>
--- a/task-reviews/puzzles/task_puzzles_spatial_cube_removal_count/task_puzzles_spatial_cube_removal_count.xlsx
+++ b/task-reviews/puzzles/task_puzzles_spatial_cube_removal_count/task_puzzles_spatial_cube_removal_count.xlsx
@@ -1792,12 +1792,12 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[108.0, 168.018, 552.0, 637.982], [648.0, 168.018, 1092.0, 637.982]], "answer": 1}</t>
+          <t>{"evidence": [[108.0, 183.277, 552.0, 622.723], [648.0, 201.587, 1092.0, 604.413]], "answer": 4}</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>[[108.0, 168.018, 552.0, 637.982], [648.0, 168.018, 1092.0, 637.982]]</t>
+          <t>[[108.0, 183.277, 552.0, 622.723], [648.0, 201.587, 1092.0, 604.413]]</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -1856,7 +1856,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[108.0, 219.897, 552.0, 586.103], [648.0, 219.897, 1092.0, 586.103]], "answer": 6}</t>
+          <t>{"evidence": [[108.0, 219.897, 552.0, 586.103], [648.0, 219.897, 1092.0, 586.103]], "answer": 5}</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1920,7 +1920,7 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[108.0, 146.656, 552.0, 659.344], [648.0, 146.656, 1092.0, 659.344]], "answer": 1}</t>
+          <t>{"evidence": [[108.0, 146.656, 552.0, 659.344], [648.0, 146.656, 1092.0, 659.344]], "answer": 2}</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
@@ -2048,12 +2048,12 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[108.0, 146.656, 552.0, 659.344], [648.0, 146.656, 1092.0, 659.344]], "answer": 2}</t>
+          <t>{"evidence": [[108.0, 189.38, 552.0, 616.62], [648.0, 189.38, 1092.0, 616.62]], "answer": 4}</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>[[108.0, 146.656, 552.0, 659.344], [648.0, 146.656, 1092.0, 659.344]]</t>
+          <t>[[108.0, 189.38, 552.0, 616.62], [648.0, 189.38, 1092.0, 616.62]]</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -2112,12 +2112,12 @@
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[202.818, 146.0, 457.182, 660.0], [742.818, 182.714, 997.182, 623.286]], "answer": 3}</t>
+          <t>{"evidence": [[202.818, 146.0, 457.182, 660.0], [742.818, 146.0, 997.182, 660.0]], "answer": 2}</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>[[202.818, 146.0, 457.182, 660.0], [742.818, 182.714, 997.182, 623.286]]</t>
+          <t>[[202.818, 146.0, 457.182, 660.0], [742.818, 146.0, 997.182, 660.0]]</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -2240,12 +2240,12 @@
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[108.0, 168.018, 552.0, 637.982], [648.0, 168.018, 1092.0, 637.982]], "answer": 2}</t>
+          <t>{"evidence": [[108.0, 219.897, 552.0, 586.103], [648.0, 238.208, 1092.0, 567.792]], "answer": 4}</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>[[108.0, 168.018, 552.0, 637.982], [648.0, 168.018, 1092.0, 637.982]]</t>
+          <t>[[108.0, 219.897, 552.0, 586.103], [648.0, 238.208, 1092.0, 567.792]]</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -2304,12 +2304,12 @@
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[108.0, 183.277, 552.0, 622.723], [648.0, 201.587, 1092.0, 604.413]], "answer": 3}</t>
+          <t>{"evidence": [[108.0, 183.277, 552.0, 622.723], [648.0, 183.277, 1092.0, 622.723]], "answer": 1}</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>[[108.0, 183.277, 552.0, 622.723], [648.0, 201.587, 1092.0, 604.413]]</t>
+          <t>[[108.0, 183.277, 552.0, 622.723], [648.0, 183.277, 1092.0, 622.723]]</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -2368,7 +2368,7 @@
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[181.621, 146.0, 478.379, 660.0], [721.621, 146.0, 1018.379, 660.0]], "answer": 2}</t>
+          <t>{"evidence": [[181.621, 146.0, 478.379, 660.0], [721.621, 146.0, 1018.379, 660.0]], "answer": 1}</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
@@ -2432,12 +2432,12 @@
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[108.0, 219.897, 552.0, 586.103], [648.0, 219.897, 1092.0, 586.103]], "answer": 1}</t>
+          <t>{"evidence": [[108.0, 201.587, 552.0, 604.413], [648.0, 219.897, 1092.0, 586.103]], "answer": 5}</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>[[108.0, 219.897, 552.0, 586.103], [648.0, 219.897, 1092.0, 586.103]]</t>
+          <t>[[108.0, 201.587, 552.0, 604.413], [648.0, 219.897, 1092.0, 586.103]]</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -2496,7 +2496,7 @@
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[108.0, 146.656, 552.0, 659.344], [648.0, 189.38, 1092.0, 616.62]], "answer": 4}</t>
+          <t>{"evidence": [[108.0, 146.656, 552.0, 659.344], [648.0, 189.38, 1092.0, 616.62]], "answer": 5}</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
@@ -2560,7 +2560,7 @@
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[127.665, 146.0, 532.335, 660.0], [667.665, 146.0, 1072.335, 660.0]], "answer": 2}</t>
+          <t>{"evidence": [[127.665, 146.0, 532.335, 660.0], [667.665, 146.0, 1072.335, 660.0]], "answer": 1}</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
@@ -2688,12 +2688,12 @@
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[108.0, 168.018, 552.0, 637.982], [648.0, 189.38, 1092.0, 616.62]], "answer": 6}</t>
+          <t>{"evidence": [[108.0, 146.656, 552.0, 659.344], [648.0, 168.018, 1092.0, 637.982]], "answer": 2}</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>[[108.0, 168.018, 552.0, 637.982], [648.0, 189.38, 1092.0, 616.62]]</t>
+          <t>[[108.0, 146.656, 552.0, 659.344], [648.0, 168.018, 1092.0, 637.982]]</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -2752,12 +2752,12 @@
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[108.0, 172.291, 552.0, 633.709], [648.0, 197.925, 1092.0, 608.075]], "answer": 1}</t>
+          <t>{"evidence": [[124.552, 146.0, 535.448, 660.0], [664.552, 185.538, 1075.448, 620.462]], "answer": 4}</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>[[108.0, 172.291, 552.0, 633.709], [648.0, 197.925, 1092.0, 608.075]]</t>
+          <t>[[124.552, 146.0, 535.448, 660.0], [664.552, 185.538, 1075.448, 620.462]]</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -2816,12 +2816,12 @@
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[108.0, 172.291, 552.0, 633.709], [648.0, 197.925, 1092.0, 608.075]], "answer": 2}</t>
+          <t>{"evidence": [[108.0, 168.018, 552.0, 637.982], [648.0, 168.018, 1092.0, 637.982]], "answer": 4}</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>[[108.0, 172.291, 552.0, 633.709], [648.0, 197.925, 1092.0, 608.075]]</t>
+          <t>[[108.0, 168.018, 552.0, 637.982], [648.0, 168.018, 1092.0, 637.982]]</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -2880,7 +2880,7 @@
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[108.0, 201.587, 552.0, 604.413], [648.0, 219.897, 1092.0, 586.103]], "answer": 3}</t>
+          <t>{"evidence": [[108.0, 201.587, 552.0, 604.413], [648.0, 219.897, 1092.0, 586.103]], "answer": 2}</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
@@ -2944,7 +2944,7 @@
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[108.0, 219.897, 552.0, 586.103], [648.0, 219.897, 1092.0, 586.103]], "answer": 3}</t>
+          <t>{"evidence": [[108.0, 219.897, 552.0, 586.103], [648.0, 219.897, 1092.0, 586.103]], "answer": 1}</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
@@ -3008,12 +3008,12 @@
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[108.0, 201.587, 552.0, 604.413], [648.0, 219.897, 1092.0, 586.103]], "answer": 6}</t>
+          <t>{"evidence": [[108.0, 146.656, 552.0, 659.344], [648.0, 197.925, 1092.0, 608.075]], "answer": 3}</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>[[108.0, 201.587, 552.0, 604.413], [648.0, 219.897, 1092.0, 586.103]]</t>
+          <t>[[108.0, 146.656, 552.0, 659.344], [648.0, 197.925, 1092.0, 608.075]]</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
@@ -3136,12 +3136,12 @@
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[108.0, 219.897, 552.0, 586.103], [648.0, 219.897, 1092.0, 586.103]], "answer": 3}</t>
+          <t>{"evidence": [[108.0, 183.277, 552.0, 622.723], [648.0, 201.587, 1092.0, 604.413]], "answer": 4}</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>[[108.0, 219.897, 552.0, 586.103], [648.0, 219.897, 1092.0, 586.103]]</t>
+          <t>[[108.0, 183.277, 552.0, 622.723], [648.0, 201.587, 1092.0, 604.413]]</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
@@ -3200,7 +3200,7 @@
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[108.0, 168.018, 552.0, 637.982], [648.0, 168.018, 1092.0, 637.982]], "answer": 4}</t>
+          <t>{"evidence": [[108.0, 168.018, 552.0, 637.982], [648.0, 168.018, 1092.0, 637.982]], "answer": 5}</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr">
@@ -3264,12 +3264,12 @@
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[108.0, 210.742, 552.0, 595.258], [648.0, 232.104, 1092.0, 573.896]], "answer": 2}</t>
+          <t>{"evidence": [[108.0, 219.897, 552.0, 586.103], [648.0, 238.208, 1092.0, 567.792]], "answer": 5}</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>[[108.0, 210.742, 552.0, 595.258], [648.0, 232.104, 1092.0, 573.896]]</t>
+          <t>[[108.0, 219.897, 552.0, 586.103], [648.0, 238.208, 1092.0, 567.792]]</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
@@ -3328,12 +3328,12 @@
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[108.0, 189.38, 552.0, 616.62], [648.0, 232.104, 1092.0, 573.896]], "answer": 6}</t>
+          <t>{"evidence": [[181.621, 146.0, 478.379, 660.0], [721.621, 188.833, 1018.379, 617.167]], "answer": 2}</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>[[108.0, 189.38, 552.0, 616.62], [648.0, 232.104, 1092.0, 573.896]]</t>
+          <t>[[181.621, 146.0, 478.379, 660.0], [721.621, 188.833, 1018.379, 617.167]]</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">

</xml_diff>